<commit_message>
feat(financeiro): atualizar planilha modelo oficial de contas a pagar com novo modelo Confianca
</commit_message>
<xml_diff>
--- a/public/modelos/Contas_a_Pagar.xlsx
+++ b/public/modelos/Contas_a_Pagar.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tsuna\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tsuna\Desktop\Projetos\Sistema ERP\modelos importacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11803046-0923-4E9B-9571-FEECF1986DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40808E59-DC99-4B25-84B7-960FD50B1923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$H$2725</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -66,6 +69,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -103,9 +109,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -386,17 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J269"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="56.140625" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" customWidth="1"/>
     <col min="6" max="6" width="27.7109375" customWidth="1"/>
     <col min="7" max="7" width="27.28515625" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -428,7 +439,20 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J8" s="1"/>
     </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D51" s="4"/>
+    </row>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D52" s="4"/>
+    </row>
+    <row r="269" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E269" s="1"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:H2725" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(financeiro): restaurar modelo de contas a pagar e implementar importador Excel para contas a receber
</commit_message>
<xml_diff>
--- a/public/modelos/Contas_a_Pagar.xlsx
+++ b/public/modelos/Contas_a_Pagar.xlsx
@@ -5,19 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tsuna\Desktop\Projetos\Sistema ERP\modelos importacao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tsuna\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40808E59-DC99-4B25-84B7-960FD50B1923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11803046-0923-4E9B-9571-FEECF1986DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$H$2725</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -69,9 +66,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -109,14 +103,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,17 +386,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J269"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="56.140625" customWidth="1"/>
-    <col min="2" max="2" width="40.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="30.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" customWidth="1"/>
     <col min="6" max="6" width="27.7109375" customWidth="1"/>
     <col min="7" max="7" width="27.28515625" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -439,20 +428,7 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J8" s="1"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E16" s="1"/>
-    </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D51" s="4"/>
-    </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D52" s="4"/>
-    </row>
-    <row r="269" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E269" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H2725" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(modelos): repaginar modelos de importacao com todos os campos e orientacoes
</commit_message>
<xml_diff>
--- a/public/modelos/Contas_a_Pagar.xlsx
+++ b/public/modelos/Contas_a_Pagar.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Contas a Pagar" sheetId="1" r:id="rId1"/>
+    <sheet name="Orientações" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,17 +398,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K6"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
-    <col min="8" max="8" width="28.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="32.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -427,27 +430,33 @@
         <v>Data de Pagamento</v>
       </c>
       <c r="F1" t="str">
-        <v>Veículo</v>
+        <v>Forma de Pagamento</v>
       </c>
       <c r="G1" t="str">
         <v>Caixa / Ponto de Pagamento</v>
       </c>
       <c r="H1" t="str">
+        <v>Veículo (Placa)</v>
+      </c>
+      <c r="I1" t="str">
         <v>Favorecido / Fornecedor</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Status</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Observações</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Abastecimento Semanal</v>
+        <v>Abastecimento Semanal - Frota</v>
       </c>
       <c r="B2" t="str">
         <v>Combustível</v>
       </c>
-      <c r="C2">
-        <v>250</v>
+      <c r="C2" t="str">
+        <v>250,00</v>
       </c>
       <c r="D2" t="str">
         <v>20/10/2026</v>
@@ -456,27 +465,33 @@
         <v>20/10/2026</v>
       </c>
       <c r="F2" t="str">
-        <v>ABC-1234</v>
+        <v>Cartão de Débito</v>
       </c>
       <c r="G2" t="str">
         <v>Caixa Operacional</v>
       </c>
       <c r="H2" t="str">
+        <v>ABC-1234</v>
+      </c>
+      <c r="I2" t="str">
         <v>Posto Ipiranga</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Pago</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Gasolina comum 45L</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Troca de Óleo</v>
+        <v>Troca de Óleo e Filtros</v>
       </c>
       <c r="B3" t="str">
         <v>Manutenção Veicular</v>
       </c>
-      <c r="C3">
-        <v>180</v>
+      <c r="C3" t="str">
+        <v>180,00</v>
       </c>
       <c r="D3" t="str">
         <v>25/10/2026</v>
@@ -485,27 +500,33 @@
         <v/>
       </c>
       <c r="F3" t="str">
+        <v>Pix</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Conta Bancária</v>
+      </c>
+      <c r="H3" t="str">
         <v>XYZ-9876</v>
       </c>
-      <c r="G3" t="str">
-        <v>Conta Corrente</v>
-      </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Oficina do Zé</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Pendente</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Revisão preventiva de 50.000 km</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Aquisição de EPIs</v>
+        <v>Aquisição de EPIs e Uniformes</v>
       </c>
       <c r="B4" t="str">
         <v>Segurança</v>
       </c>
-      <c r="C4">
-        <v>320</v>
+      <c r="C4" t="str">
+        <v>320,00</v>
       </c>
       <c r="D4" t="str">
         <v>15/10/2026</v>
@@ -514,21 +535,319 @@
         <v>14/10/2026</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>Boleto Bancário</v>
       </c>
       <c r="G4" t="str">
         <v>Caixa Operacional</v>
       </c>
       <c r="H4" t="str">
-        <v>Distribuidora Proteção</v>
+        <v/>
       </c>
       <c r="I4" t="str">
+        <v>Distribuidora Proteção Total</v>
+      </c>
+      <c r="J4" t="str">
         <v>Pago</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Luvas, óculos de proteção e botas para técnicos</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Aluguel do Galpão Operacional</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Instalações</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2800,00</v>
+      </c>
+      <c r="D5" t="str">
+        <v>05/11/2026</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v>Transferência</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Conta Bancária</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Imobiliária Aliança</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Pendente</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Referente ao mês de Outubro/2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Energia Elétrica e Internet Fibra</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Utilidades</v>
+      </c>
+      <c r="C6" t="str">
+        <v>430,00</v>
+      </c>
+      <c r="D6" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="E6" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Pix</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Conta Bancária</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Neoenergia / Provedor Fibra</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Contas pagas com comprovante arquivado</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E12"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="65.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Campo / Coluna</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Obrigatório?</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Tipo de Dado</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Exemplo</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Regras e Recomendações do Sistema</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Descrição da Despesa</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SIM</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Abastecimento Semanal</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Identificação ou nome da despesa/conta a pagar.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Categoria</v>
+      </c>
+      <c r="B3" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Combustível, Manutenção</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Categoria da despesa. Se não existir no sistema, será criada automaticamente.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Valor (R$)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SIM</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Numérico / Moeda</v>
+      </c>
+      <c r="D4" t="str">
+        <v>250,00 ou 250</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Valor em Reais a pagar. Aceita vírgula ou ponto (ex: 250,50 ou 250.50).</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Vencimento</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SIM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Data (DD/MM/AAAA)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>20/10/2026</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Data de vencimento da fatura ou boleto.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Data de Pagamento</v>
+      </c>
+      <c r="B6" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Data (DD/MM/AAAA)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>20/10/2026</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Data em que o pagamento foi realizado. Se deixada em branco, assume a data de vencimento.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Forma de Pagamento</v>
+      </c>
+      <c r="B7" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Pix, Boleto, Cartão</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Forma ou método de liquidação utilizado.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Caixa / Ponto de Pagamento</v>
+      </c>
+      <c r="B8" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Caixa Operacional, Conta Bancária</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Caixa de onde os recursos saíram para quitar a despesa.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Veículo (Placa)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Texto (Placa)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>ABC-1234</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Placa do veículo cadastrado na frota (opcional, para despesas automotivas).</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Favorecido / Fornecedor</v>
+      </c>
+      <c r="B10" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Posto Ipiranga</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Nome da empresa fornecedora ou pessoa que recebeu o pagamento.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B11" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Pago, Pendente ou Cancelado</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Status atual da despesa. Padrão é "Pendente" (ou "Pago" se quitada).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Observações</v>
+      </c>
+      <c r="B12" t="str">
+        <v>NÃO</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Texto</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Revisão de 50.000 km</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Campo livre para anotações, notas fiscais ou detalhes adicionais.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>